<commit_message>
trying to host backend on render
</commit_message>
<xml_diff>
--- a/backend/Auto_Wrapping_Analytics.xlsx
+++ b/backend/Auto_Wrapping_Analytics.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL1"/>
+  <dimension ref="A1:AL3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,6 +605,151 @@
       <c r="AL1" t="inlineStr">
         <is>
           <t>Overweight %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Auto 9</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>odogwu</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G2" t="n">
+        <v>120</v>
+      </c>
+      <c r="H2" t="n">
+        <v>122</v>
+      </c>
+      <c r="I2" t="n">
+        <v>128</v>
+      </c>
+      <c r="J2" t="n">
+        <v>119</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>121.8</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>80.0</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Auto 9</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>gsr</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>31</v>
+      </c>
+      <c r="G3" t="n">
+        <v>32</v>
+      </c>
+      <c r="H3" t="n">
+        <v>32</v>
+      </c>
+      <c r="I3" t="n">
+        <v>32</v>
+      </c>
+      <c r="J3" t="n">
+        <v>33</v>
+      </c>
+      <c r="K3" t="n">
+        <v>33</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>32.2</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>6</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>0.0</t>
         </is>
       </c>
     </row>

</xml_diff>